<commit_message>
feat(routing): cost-aware multilingual fast router with 5k synthetic benchmark and cost model
</commit_message>
<xml_diff>
--- a/deliverables/cheerio_resolve_eval_and_cost_workbook.xlsx
+++ b/deliverables/cheerio_resolve_eval_and_cost_workbook.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Label Guide" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Evaluation Scorecard" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Cost Assumptions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Multilingual Cost Model" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Scenarios'!$A$1:$S$171</definedName>
@@ -21,8 +22,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.00000"/>
+  </numFmts>
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,8 +39,53 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00004D40"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00006100"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -47,8 +97,32 @@
         <fgColor rgb="00243B53"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE6F1"/>
+        <bgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F497D"/>
+        <bgColor rgb="001F497D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -56,17 +130,141 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="double">
+        <color rgb="001F497D"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -16910,7 +17108,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>100</v>
+        <v>5000</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -16919,17 +17117,17 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>ASSUMPTION</t>
+          <t>[ASSUMPTION]</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>User-editable</t>
+          <t>Target business scale benchmark</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Replace with sourced estimate.</t>
+          <t>Scale baseline for 5,000 active merchant businesses</t>
         </is>
       </c>
     </row>
@@ -17060,7 +17258,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>0</v>
+        <v>0.59</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -17069,17 +17267,17 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>TO VERIFY</t>
+          <t>[DOCUMENTED]</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Provider pricing page + access date</t>
+          <t>Groq Llama-3.3-70b-versatile public pricing</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Use current public pricing only after browser-use verification.</t>
+          <t>USD per 1M prompt/input tokens (accessed 2024-10)</t>
         </is>
       </c>
     </row>
@@ -17090,7 +17288,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>0</v>
+        <v>0.79</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
@@ -17099,17 +17297,17 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>TO VERIFY</t>
+          <t>[DOCUMENTED]</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Provider pricing page + access date</t>
+          <t>Groq Llama-3.3-70b-versatile public pricing</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Use current public pricing only after browser-use verification.</t>
+          <t>USD per 1M completion/output tokens (accessed 2024-10)</t>
         </is>
       </c>
     </row>
@@ -17120,7 +17318,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>1200</v>
+        <v>450</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -17129,12 +17327,12 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>ASSUMPTION</t>
+          <t>[SYNTHETIC BENCHMARK]</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>User-editable</t>
+          <t>Single-turn structured intent fallback prompt</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -17150,7 +17348,7 @@
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
@@ -17159,12 +17357,12 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>ASSUMPTION</t>
+          <t>[SYNTHETIC BENCHMARK]</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>User-editable</t>
+          <t>Structured JSON interpretation payload</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -17362,4 +17560,1135 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Cheerio Resolve — Multilingual Fast Router &amp; Scaled Cost Model</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>5,000 Active Businesses Workload Analysis across English, Hinglish, Devanagari Hindi, and Mixed Scripts</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Metric / Model Parameter</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Unit / Basis</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Low Activity</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Base Case</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>High Activity</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Evidence Label</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Source / Methodology / Formula Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>1. Business Scale &amp; Support Volume (5,000 Active Businesses)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Active businesses on platform</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>businesses</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>[ASSUMPTION]</t>
+        </is>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>Scale target: 5,000 merchant businesses using WhatsApp customer channels</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>Monthly customer support messages per business</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>messages / biz / month</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>60</v>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>[ASSUMPTION]</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Low: 10 (early onboarding); Base: 25 (steady-state); High: 60 (festival/peak season)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Total monthly support messages evaluated</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>messages / month</t>
+        </is>
+      </c>
+      <c r="C8" s="13">
+        <f>C6*C7</f>
+        <v/>
+      </c>
+      <c r="D8" s="13">
+        <f>D6*D7</f>
+        <v/>
+      </c>
+      <c r="E8" s="13">
+        <f>E6*E7</f>
+        <v/>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>[FORMULA]</t>
+        </is>
+      </c>
+      <c r="G8" s="12">
+        <f> Businesses × Monthly messages per business</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>2. Multilingual Router Performance (5,000 Synthetic Benchmark)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Deterministic Fast Router share (Layer 1: 0 LLM calls)</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>routing %</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="n">
+        <v>0.8536</v>
+      </c>
+      <c r="D10" s="15" t="n">
+        <v>0.8536</v>
+      </c>
+      <c r="E10" s="15" t="n">
+        <v>0.8536</v>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>[SYNTHETIC BENCHMARK]</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>Sub-millisecond regex fast router in domain layer (measured on 5,000 synthetic messages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="9" t="inlineStr">
+        <is>
+          <t>Ambiguous / Novel fallback share (Layer 2: Groq LLM)</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>routing %</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>0.1464</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <v>0.1464</v>
+      </c>
+      <c r="E11" s="15" t="n">
+        <v>0.1464</v>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>[SYNTHETIC BENCHMARK]</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Messages requiring single structured LLM fallback (no separate translation call)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Deterministic messages resolved without LLM</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>messages / month</t>
+        </is>
+      </c>
+      <c r="C12" s="17">
+        <f>C8*C10</f>
+        <v/>
+      </c>
+      <c r="D12" s="17">
+        <f>D8*D10</f>
+        <v/>
+      </c>
+      <c r="E12" s="17">
+        <f>E8*E10</f>
+        <v/>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>[FORMULA]</t>
+        </is>
+      </c>
+      <c r="G12" s="16">
+        <f> Total monthly messages × Deterministic Fast Router share</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Ambiguous messages routed to hosted LLM</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>queries / month</t>
+        </is>
+      </c>
+      <c r="C13" s="17">
+        <f>C8*C11</f>
+        <v/>
+      </c>
+      <c r="D13" s="17">
+        <f>D8*D11</f>
+        <v/>
+      </c>
+      <c r="E13" s="17">
+        <f>E8*E11</f>
+        <v/>
+      </c>
+      <c r="F13" s="18" t="inlineStr">
+        <is>
+          <t>[FORMULA]</t>
+        </is>
+      </c>
+      <c r="G13" s="16">
+        <f> Total monthly messages × LLM fallback share</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>LLM JSON schema parsing retry buffer</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>retry rate %</t>
+        </is>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>[ASSUMPTION]</t>
+        </is>
+      </c>
+      <c r="G14" s="9" t="inlineStr">
+        <is>
+          <t>2.0% buffer for rare schema retry when JSON parsing fails</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Net billable LLM fallback calls per month</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>calls / month</t>
+        </is>
+      </c>
+      <c r="C15" s="13">
+        <f>C13*(1+C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="13">
+        <f>D13*(1+D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="13">
+        <f>E13*(1+E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>[FORMULA]</t>
+        </is>
+      </c>
+      <c r="G15" s="12">
+        <f> Ambiguous queries × (1 + Retry rate)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>Fast router average latency per message</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>milliseconds</t>
+        </is>
+      </c>
+      <c r="C16" s="19" t="n">
+        <v>0.0245</v>
+      </c>
+      <c r="D16" s="19" t="n">
+        <v>0.0245</v>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>0.0245</v>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>[SYNTHETIC BENCHMARK]</t>
+        </is>
+      </c>
+      <c r="G16" s="9" t="inlineStr">
+        <is>
+          <t>Measured in-process memory regex lookup (sub-millisecond target passed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Fast router p99 latency per message</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>milliseconds</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="n">
+        <v>0.0741</v>
+      </c>
+      <c r="D17" s="19" t="n">
+        <v>0.0741</v>
+      </c>
+      <c r="E17" s="19" t="n">
+        <v>0.0741</v>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>[SYNTHETIC BENCHMARK]</t>
+        </is>
+      </c>
+      <c r="G17" s="9" t="inlineStr">
+        <is>
+          <t>99th percentile response time for deterministic router</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>Critical safety violations in benchmark</t>
+        </is>
+      </c>
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>violations</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="22" t="inlineStr">
+        <is>
+          <t>[SYNTHETIC BENCHMARK]</t>
+        </is>
+      </c>
+      <c r="G18" s="20" t="inlineStr">
+        <is>
+          <t>Zero safety violations: Billing (G10), Security (G10) &amp; human requests escalated</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>3. Token Economics &amp; Provider Rates (Groq Llama-3.3-70b-versatile)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Groq input prompt pricing</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>USD / 1M tokens</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="D20" s="23" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="E20" s="23" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>[DOCUMENTED]</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Official Groq cloud pricing for Llama-3.3-70b-versatile</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Groq output completion pricing</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>USD / 1M tokens</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="D21" s="23" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="E21" s="23" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="F21" s="11" t="inlineStr">
+        <is>
+          <t>[DOCUMENTED]</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>Official Groq cloud pricing for Llama-3.3-70b-versatile</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Average input tokens per structured interpretation</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>tokens / request</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>450</v>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>450</v>
+      </c>
+      <c r="E22" s="10" t="n">
+        <v>450</v>
+      </c>
+      <c r="F22" s="11" t="inlineStr">
+        <is>
+          <t>[SYNTHETIC BENCHMARK]</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>Single-turn prompt with intent schemas, language rules and context</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Average output tokens per structured interpretation</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>tokens / request</t>
+        </is>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="E23" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="F23" s="11" t="inlineStr">
+        <is>
+          <t>[SYNTHETIC BENCHMARK]</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>Structured JSON with intent, language, entities, explanation &amp; next step</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Estimated blended cost per LLM fallback call</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>USD / call</t>
+        </is>
+      </c>
+      <c r="C24" s="24">
+        <f>(C22*C20/1000000)+(C23*C21/1000000)</f>
+        <v/>
+      </c>
+      <c r="D24" s="24">
+        <f>(D22*D20/1000000)+(D23*D21/1000000)</f>
+        <v/>
+      </c>
+      <c r="E24" s="24">
+        <f>(E22*E20/1000000)+(E23*E21/1000000)</f>
+        <v/>
+      </c>
+      <c r="F24" s="14" t="inlineStr">
+        <is>
+          <t>[FORMULA]</t>
+        </is>
+      </c>
+      <c r="G24" s="12">
+        <f> (Input tokens × Input price / 1M) + (Output tokens × Output price / 1M)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>4. Monthly Operating Cost Comparison (Pure LLM vs Totoro Fast Router)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Architecture A: Pure 100% LLM Routing (No Fast Router)</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>calls / month</t>
+        </is>
+      </c>
+      <c r="C26" s="10">
+        <f>C8*(1+C14)</f>
+        <v/>
+      </c>
+      <c r="D26" s="10">
+        <f>D8*(1+D14)</f>
+        <v/>
+      </c>
+      <c r="E26" s="10">
+        <f>E8*(1+E14)</f>
+        <v/>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>[FORMULA]</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>Every single support turn calls Groq LLM (with 2% retry buffer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="25" t="inlineStr">
+        <is>
+          <t>Architecture A: Total monthly LLM cost</t>
+        </is>
+      </c>
+      <c r="B27" s="25" t="inlineStr">
+        <is>
+          <t>USD / month</t>
+        </is>
+      </c>
+      <c r="C27" s="26">
+        <f>C26*C24</f>
+        <v/>
+      </c>
+      <c r="D27" s="26">
+        <f>D26*D24</f>
+        <v/>
+      </c>
+      <c r="E27" s="26">
+        <f>E26*E24</f>
+        <v/>
+      </c>
+      <c r="F27" s="27" t="inlineStr">
+        <is>
+          <t>[FORMULA]</t>
+        </is>
+      </c>
+      <c r="G27" s="25">
+        <f> Architecture A calls × Cost per call</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Architecture B: Totoro Hybrid (Fast Router + LLM Fallback)</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>calls / month</t>
+        </is>
+      </c>
+      <c r="C28" s="10">
+        <f>C15</f>
+        <v/>
+      </c>
+      <c r="D28" s="10">
+        <f>D15</f>
+        <v/>
+      </c>
+      <c r="E28" s="10">
+        <f>E15</f>
+        <v/>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>[FORMULA]</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>Only ambiguous/novel queries reach LLM (85.36% resolved deterministically)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="28" t="inlineStr">
+        <is>
+          <t>Architecture B: Total monthly LLM cost</t>
+        </is>
+      </c>
+      <c r="B29" s="28" t="inlineStr">
+        <is>
+          <t>USD / month</t>
+        </is>
+      </c>
+      <c r="C29" s="29">
+        <f>C28*C24</f>
+        <v/>
+      </c>
+      <c r="D29" s="29">
+        <f>D28*D24</f>
+        <v/>
+      </c>
+      <c r="E29" s="29">
+        <f>E28*E24</f>
+        <v/>
+      </c>
+      <c r="F29" s="30" t="inlineStr">
+        <is>
+          <t>[FORMULA]</t>
+        </is>
+      </c>
+      <c r="G29" s="28">
+        <f> Architecture B calls × Cost per call</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="20" t="inlineStr">
+        <is>
+          <t>Net Monthly Dollar Savings with Fast Router</t>
+        </is>
+      </c>
+      <c r="B30" s="20" t="inlineStr">
+        <is>
+          <t>USD / month</t>
+        </is>
+      </c>
+      <c r="C30" s="31">
+        <f>C27-C29</f>
+        <v/>
+      </c>
+      <c r="D30" s="31">
+        <f>D27-D29</f>
+        <v/>
+      </c>
+      <c r="E30" s="31">
+        <f>E27-E29</f>
+        <v/>
+      </c>
+      <c r="F30" s="22" t="inlineStr">
+        <is>
+          <t>[FORMULA]</t>
+        </is>
+      </c>
+      <c r="G30" s="20">
+        <f> Architecture A cost - Architecture B cost</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="20" t="inlineStr">
+        <is>
+          <t>Net Annual Dollar Savings with Fast Router</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="inlineStr">
+        <is>
+          <t>USD / year</t>
+        </is>
+      </c>
+      <c r="C31" s="31">
+        <f>C30*12</f>
+        <v/>
+      </c>
+      <c r="D31" s="31">
+        <f>D30*12</f>
+        <v/>
+      </c>
+      <c r="E31" s="31">
+        <f>E30*12</f>
+        <v/>
+      </c>
+      <c r="F31" s="22" t="inlineStr">
+        <is>
+          <t>[FORMULA]</t>
+        </is>
+      </c>
+      <c r="G31" s="20">
+        <f> Monthly savings × 12 months</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="32" t="inlineStr">
+        <is>
+          <t>Cost Reduction Percentage</t>
+        </is>
+      </c>
+      <c r="B32" s="32" t="inlineStr">
+        <is>
+          <t>% reduction</t>
+        </is>
+      </c>
+      <c r="C32" s="33">
+        <f>(C27-C29)/C27</f>
+        <v/>
+      </c>
+      <c r="D32" s="33">
+        <f>(D27-D29)/D27</f>
+        <v/>
+      </c>
+      <c r="E32" s="33">
+        <f>(E27-E29)/E27</f>
+        <v/>
+      </c>
+      <c r="F32" s="34" t="inlineStr">
+        <is>
+          <t>[FORMULA]</t>
+        </is>
+      </c>
+      <c r="G32" s="32">
+        <f> (Pure LLM cost - Totoro cost) / Pure LLM cost</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>5. Workload Language Breakdown (Observed Synthetic Distribution)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>English language queries (40.0%)</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>messages / month</t>
+        </is>
+      </c>
+      <c r="C34" s="10">
+        <f>C8*0.40</f>
+        <v/>
+      </c>
+      <c r="D34" s="10">
+        <f>D8*0.40</f>
+        <v/>
+      </c>
+      <c r="E34" s="10">
+        <f>E8*0.40</f>
+        <v/>
+      </c>
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>[SYNTHETIC BENCHMARK]</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>40.0% of synthetic support dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>Hinglish / Romanized Hindi queries (35.0%)</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>messages / month</t>
+        </is>
+      </c>
+      <c r="C35" s="10">
+        <f>C8*0.35</f>
+        <v/>
+      </c>
+      <c r="D35" s="10">
+        <f>D8*0.35</f>
+        <v/>
+      </c>
+      <c r="E35" s="10">
+        <f>E8*0.35</f>
+        <v/>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
+        <is>
+          <t>[SYNTHETIC BENCHMARK]</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>35.0% of synthetic support dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>Devanagari Hindi script queries (15.0%)</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>messages / month</t>
+        </is>
+      </c>
+      <c r="C36" s="10">
+        <f>C8*0.15</f>
+        <v/>
+      </c>
+      <c r="D36" s="10">
+        <f>D8*0.15</f>
+        <v/>
+      </c>
+      <c r="E36" s="10">
+        <f>E8*0.15</f>
+        <v/>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>[SYNTHETIC BENCHMARK]</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="inlineStr">
+        <is>
+          <t>15.0% of synthetic support dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>Mixed-script (Latin + Devanagari) queries (10.0%)</t>
+        </is>
+      </c>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>messages / month</t>
+        </is>
+      </c>
+      <c r="C37" s="10">
+        <f>C8*0.10</f>
+        <v/>
+      </c>
+      <c r="D37" s="10">
+        <f>D8*0.10</f>
+        <v/>
+      </c>
+      <c r="E37" s="10">
+        <f>E8*0.10</f>
+        <v/>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
+        <is>
+          <t>[SYNTHETIC BENCHMARK]</t>
+        </is>
+      </c>
+      <c r="G37" s="9" t="inlineStr">
+        <is>
+          <t>10.0% of synthetic support dataset</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>6. Human Escalation &amp; Containment Safety (G8–G12 Guardrails)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>Policy &amp; guardrail human escalation rate</t>
+        </is>
+      </c>
+      <c r="B39" s="9" t="inlineStr">
+        <is>
+          <t>escalation %</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="n">
+        <v>0.1448</v>
+      </c>
+      <c r="D39" s="15" t="n">
+        <v>0.1448</v>
+      </c>
+      <c r="E39" s="15" t="n">
+        <v>0.1448</v>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>[SYNTHETIC BENCHMARK]</t>
+        </is>
+      </c>
+      <c r="G39" s="9" t="inlineStr">
+        <is>
+          <t>Mandatory human-led zones: Billing/refunds, security/passwords, human agent requests</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>Estimated human specialist handoffs generated</t>
+        </is>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>handoffs / month</t>
+        </is>
+      </c>
+      <c r="C40" s="17">
+        <f>C8*C39</f>
+        <v/>
+      </c>
+      <c r="D40" s="17">
+        <f>D8*D39</f>
+        <v/>
+      </c>
+      <c r="E40" s="17">
+        <f>E8*E39</f>
+        <v/>
+      </c>
+      <c r="F40" s="18" t="inlineStr">
+        <is>
+          <t>[FORMULA]</t>
+        </is>
+      </c>
+      <c r="G40" s="16" t="inlineStr">
+        <is>
+          <t>Escalated to human support queue with complete pre-populated case file</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>Automated self-service containment</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>resolutions / month</t>
+        </is>
+      </c>
+      <c r="C41" s="13">
+        <f>C8-C40</f>
+        <v/>
+      </c>
+      <c r="D41" s="13">
+        <f>D8-D40</f>
+        <v/>
+      </c>
+      <c r="E41" s="13">
+        <f>E8-E40</f>
+        <v/>
+      </c>
+      <c r="F41" s="14" t="inlineStr">
+        <is>
+          <t>[FORMULA]</t>
+        </is>
+      </c>
+      <c r="G41" s="12" t="inlineStr">
+        <is>
+          <t>Handled end-to-end by Totoro's playbook verification and consent flow</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A5:G5"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>